<commit_message>
Product image and names updated.
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\crystal-code\python-util\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ejasaki\project\python-util\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C66F09-95EF-4AC4-AA3C-61C06E0DED40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="11496"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bracelets" sheetId="1" r:id="rId1"/>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="157">
   <si>
     <t>BR0001</t>
   </si>
@@ -302,9 +303,6 @@
     <t>BR0039</t>
   </si>
   <si>
-    <t>ROHDONITE</t>
-  </si>
-  <si>
     <t>BR0041</t>
   </si>
   <si>
@@ -380,9 +378,6 @@
     <t>DC0007</t>
   </si>
   <si>
-    <t>SMALL TREE</t>
-  </si>
-  <si>
     <t>HL0001</t>
   </si>
   <si>
@@ -392,9 +387,6 @@
     <t>HL0002</t>
   </si>
   <si>
-    <t>ANGEL STICKS</t>
-  </si>
-  <si>
     <t>HL0003</t>
   </si>
   <si>
@@ -498,12 +490,24 @@
   </si>
   <si>
     <t>BR0023B</t>
+  </si>
+  <si>
+    <t>TIGER EYE A+++</t>
+  </si>
+  <si>
+    <t>TIGER EYE TREE (SMALL)</t>
+  </si>
+  <si>
+    <t>TOURMALINE HEALING STICK (ANGEL)</t>
+  </si>
+  <si>
+    <t>RHODONITE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -561,7 +565,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -569,14 +573,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -857,16 +855,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C82"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.21875" customWidth="1"/>
-    <col min="2" max="2" width="21.44140625" customWidth="1"/>
-    <col min="3" max="3" width="12.109375" customWidth="1"/>
+    <col min="1" max="1" width="12.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.453125" customWidth="1"/>
+    <col min="3" max="3" width="12.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -877,530 +875,530 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="5"/>
-    </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="5"/>
-    </row>
-    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="5"/>
-    </row>
-    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="5"/>
-    </row>
-    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="5"/>
-    </row>
-    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="5"/>
-    </row>
-    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="5"/>
-    </row>
-    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="5"/>
-    </row>
-    <row r="12" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="5"/>
-    </row>
-    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="5"/>
-    </row>
-    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="5"/>
-    </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="5"/>
-    </row>
-    <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C16" s="5"/>
-    </row>
-    <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="5"/>
-    </row>
-    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C18" s="5"/>
-    </row>
-    <row r="19" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C19" s="5"/>
-    </row>
-    <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C20" s="5"/>
-    </row>
-    <row r="21" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C21" s="5"/>
-    </row>
-    <row r="22" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="4" t="s">
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="5"/>
-    </row>
-    <row r="23" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="4" t="s">
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C23" s="5"/>
-    </row>
-    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
+      <c r="C23" s="2"/>
+    </row>
+    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="5"/>
-    </row>
-    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="B25" s="4" t="s">
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C25" s="5"/>
-    </row>
-    <row r="26" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="B26" s="4" t="s">
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="4"/>
-    </row>
-    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="4" t="s">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C27" s="5"/>
-    </row>
-    <row r="28" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="4" t="s">
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C28" s="5"/>
-    </row>
-    <row r="29" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="4" t="s">
+      <c r="C28" s="2"/>
+    </row>
+    <row r="29" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C29" s="5"/>
-    </row>
-    <row r="30" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="4" t="s">
+      <c r="C29" s="2"/>
+    </row>
+    <row r="30" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C30" s="5"/>
-    </row>
-    <row r="31" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="4" t="s">
+      <c r="C30" s="2"/>
+    </row>
+    <row r="31" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C31" s="5"/>
-    </row>
-    <row r="32" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="4" t="s">
+      <c r="C31" s="2"/>
+    </row>
+    <row r="32" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C32" s="5"/>
-    </row>
-    <row r="33" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="4" t="s">
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A33" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="5"/>
-    </row>
-    <row r="34" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="4" t="s">
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C34" s="5"/>
-    </row>
-    <row r="35" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="4" t="s">
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C35" s="5"/>
-    </row>
-    <row r="36" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="4" t="s">
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C36" s="5"/>
-    </row>
-    <row r="37" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="4" t="s">
+      <c r="C36" s="2"/>
+    </row>
+    <row r="37" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C37" s="5"/>
-    </row>
-    <row r="38" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="4" t="s">
+      <c r="C37" s="2"/>
+    </row>
+    <row r="38" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C38" s="5"/>
-    </row>
-    <row r="39" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="4" t="s">
+      <c r="C38" s="2"/>
+    </row>
+    <row r="39" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A39" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C39" s="5"/>
-    </row>
-    <row r="40" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="4" t="s">
+      <c r="C39" s="2"/>
+    </row>
+    <row r="40" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A40" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C40" s="5"/>
-    </row>
-    <row r="41" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="4" t="s">
+      <c r="C40" s="2"/>
+    </row>
+    <row r="41" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A41" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C41" s="5"/>
-    </row>
-    <row r="42" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="4" t="s">
+      <c r="C41" s="2"/>
+    </row>
+    <row r="42" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A42" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C42" s="5"/>
-    </row>
-    <row r="43" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="4" t="s">
+      <c r="C42" s="2"/>
+    </row>
+    <row r="43" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A43" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B43" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C43" s="2"/>
+    </row>
+    <row r="44" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A44" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C44" s="2"/>
+    </row>
+    <row r="45" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A45" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C43" s="5"/>
-    </row>
-    <row r="44" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C44" s="5"/>
-    </row>
-    <row r="45" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="4" t="s">
+      <c r="B45" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="C45" s="2"/>
+    </row>
+    <row r="46" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A46" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C46" s="2"/>
+    </row>
+    <row r="47" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A47" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C45" s="5"/>
-    </row>
-    <row r="46" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C46" s="5"/>
-    </row>
-    <row r="47" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="4" t="s">
+      <c r="B47" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="C47" s="1"/>
+    </row>
+    <row r="48" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A48" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48" s="2"/>
+    </row>
+    <row r="49" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A49" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C47" s="4"/>
-    </row>
-    <row r="48" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C48" s="5"/>
-    </row>
-    <row r="49" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="4" t="s">
+      <c r="B49" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C49" s="5"/>
-    </row>
-    <row r="53" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="54" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C49" s="2"/>
+    </row>
+    <row r="53" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="54" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
     </row>
-    <row r="55" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
     </row>
-    <row r="56" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C56" s="2"/>
     </row>
-    <row r="63" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="64" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C64" s="4"/>
-    </row>
-    <row r="65" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C65" s="4"/>
-    </row>
-    <row r="66" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C66" s="4"/>
-    </row>
-    <row r="67" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C67" s="5"/>
-    </row>
-    <row r="68" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C68" s="5"/>
-    </row>
-    <row r="69" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="64" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C64" s="1"/>
+    </row>
+    <row r="65" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C65" s="1"/>
+    </row>
+    <row r="66" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C66" s="1"/>
+    </row>
+    <row r="67" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C67" s="2"/>
+    </row>
+    <row r="68" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C68" s="2"/>
+    </row>
+    <row r="69" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C69" s="2"/>
     </row>
-    <row r="70" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="2"/>
     </row>
-    <row r="71" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="2"/>
     </row>
-    <row r="72" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="2"/>
     </row>
-    <row r="73" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="2"/>
     </row>
-    <row r="74" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="2"/>
     </row>
-    <row r="75" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="2"/>
     </row>
-    <row r="76" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="2"/>
     </row>
-    <row r="77" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="2"/>
     </row>
-    <row r="78" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="2"/>
     </row>
-    <row r="79" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="2"/>
     </row>
-    <row r="80" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
     </row>
-    <row r="81" spans="3:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="3:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C81" s="1"/>
     </row>
-    <row r="82" spans="3:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="3:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C82" s="2"/>
     </row>
   </sheetData>
@@ -1410,11 +1408,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -1425,20 +1423,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="54" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="51.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -1447,11 +1445,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -1462,84 +1460,84 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="54" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="51.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B2" s="1" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="1" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="1" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="64" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="1" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="54" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B4" s="1" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="64" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="67.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B5" s="1" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="51.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="1" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="67.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B6" s="1" t="s">
+    </row>
+    <row r="8" spans="1:3" ht="76.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="1" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="54" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B7" s="1" t="s">
+    </row>
+    <row r="9" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="1" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="80.400000000000006" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B8" s="1" t="s">
+    </row>
+    <row r="10" spans="1:3" ht="51.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="B9" s="1" t="s">
+    </row>
+    <row r="11" spans="1:3" ht="51.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="54" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="54" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -1548,14 +1546,14 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="26.77734375" customWidth="1"/>
+    <col min="2" max="2" width="26.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -1566,80 +1564,84 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="5"/>
-    </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C4" s="5"/>
-    </row>
-    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+      <c r="B5" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="5"/>
-    </row>
-    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C6" s="5"/>
-    </row>
-    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
+      <c r="B7" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="5"/>
-    </row>
-    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C8" s="4"/>
+      <c r="B8" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C8" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="37.453125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -1650,68 +1652,69 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="54" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B3" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="1" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="4" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="1" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="54" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B4" s="1" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="1" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="1" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="1" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="54" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>128</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
+    <col min="2" max="2" width="26.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -1722,12 +1725,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1736,15 +1739,15 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="26.21875" defaultRowHeight="99" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="26.1796875" defaultRowHeight="99" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" customWidth="1"/>
+    <col min="1" max="1" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="16.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -1755,7 +1758,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="39" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -1764,30 +1767,30 @@
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>102</v>
       </c>
       <c r="C5" s="2"/>
     </row>

</xml_diff>